<commit_message>
feat: Enhance predicted material requirement page
</commit_message>
<xml_diff>
--- a/auto_upload/order_models/成品入庫TECO狀態.XLSX
+++ b/auto_upload/order_models/成品入庫TECO狀態.XLSX
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gfpap\june\auto_upload\order_models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{638E83FF-EB7E-4FE2-ACFC-F0F3A4DA1DA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7598CF4C-3B73-46A1-A7AB-9A1D469092B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="588" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="576" uniqueCount="209">
   <si>
     <t>ZP01</t>
   </si>
@@ -76,15 +76,6 @@
     <t>5BC-226_X=2M,Y=2.6M,Z=1.0/1.2/1.4M</t>
   </si>
   <si>
-    <t>100002943</t>
-  </si>
-  <si>
-    <t>980000038401</t>
-  </si>
-  <si>
-    <t>5A-65E_X=650,Y=520,Z=460</t>
-  </si>
-  <si>
     <t>100002954</t>
   </si>
   <si>
@@ -599,15 +590,6 @@
   </si>
   <si>
     <t>5BC-429_X=4M,Y=2.9M,Z=1.0/1.2/1.4M</t>
-  </si>
-  <si>
-    <t>100002156</t>
-  </si>
-  <si>
-    <t>980000018201</t>
-  </si>
-  <si>
-    <t>HSA-423,#50_X4000,Y2300,Z780/1070/1200</t>
   </si>
   <si>
     <t>REL  MSPT PCNF DLV  PRC  MANC RESA RMWB*</t>
@@ -1077,7 +1059,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L97"/>
+  <dimension ref="A1:L95"/>
   <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" bestFit="1" customWidth="1"/>
@@ -1093,40 +1075,40 @@
   <sheetData>
     <row r="1" spans="1:12" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="I1" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="J1" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>207</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>208</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>212</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
@@ -1134,37 +1116,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>193</v>
+        <v>3</v>
       </c>
       <c r="C2" s="2">
         <v>1</v>
       </c>
       <c r="D2" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E2" t="s">
-        <v>194</v>
+        <v>4</v>
       </c>
       <c r="F2" t="s">
-        <v>195</v>
+        <v>5</v>
       </c>
       <c r="G2" s="3">
-        <v>44902</v>
+        <v>45155</v>
       </c>
       <c r="H2" s="3">
-        <v>44921</v>
+        <v>45250</v>
       </c>
       <c r="I2" s="3">
-        <v>45077</v>
+        <v>45279</v>
       </c>
       <c r="J2" t="s">
-        <v>196</v>
+        <v>6</v>
       </c>
       <c r="K2" t="s">
         <v>1</v>
       </c>
       <c r="L2" s="3">
-        <v>44902</v>
+        <v>45152</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
@@ -1172,7 +1154,7 @@
         <v>0</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C3" s="2">
         <v>1</v>
@@ -1193,7 +1175,7 @@
         <v>45250</v>
       </c>
       <c r="I3" s="3">
-        <v>45279</v>
+        <v>45278</v>
       </c>
       <c r="J3" t="s">
         <v>6</v>
@@ -1210,7 +1192,7 @@
         <v>0</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C4" s="2">
         <v>1</v>
@@ -1248,7 +1230,7 @@
         <v>0</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C5" s="2">
         <v>1</v>
@@ -1269,7 +1251,7 @@
         <v>45250</v>
       </c>
       <c r="I5" s="3">
-        <v>45278</v>
+        <v>45279</v>
       </c>
       <c r="J5" t="s">
         <v>6</v>
@@ -1286,7 +1268,7 @@
         <v>0</v>
       </c>
       <c r="B6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C6" s="2">
         <v>1</v>
@@ -1307,7 +1289,7 @@
         <v>45250</v>
       </c>
       <c r="I6" s="3">
-        <v>45279</v>
+        <v>45278</v>
       </c>
       <c r="J6" t="s">
         <v>6</v>
@@ -1323,8 +1305,8 @@
       <c r="A7" t="s">
         <v>0</v>
       </c>
-      <c r="B7" t="s">
-        <v>10</v>
+      <c r="B7" s="5" t="s">
+        <v>208</v>
       </c>
       <c r="C7" s="2">
         <v>1</v>
@@ -1345,7 +1327,7 @@
         <v>45250</v>
       </c>
       <c r="I7" s="3">
-        <v>45278</v>
+        <v>45279</v>
       </c>
       <c r="J7" t="s">
         <v>6</v>
@@ -1361,8 +1343,8 @@
       <c r="A8" t="s">
         <v>0</v>
       </c>
-      <c r="B8" s="5" t="s">
-        <v>214</v>
+      <c r="B8" t="s">
+        <v>11</v>
       </c>
       <c r="C8" s="2">
         <v>1</v>
@@ -1371,28 +1353,28 @@
         <v>0</v>
       </c>
       <c r="E8" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="F8" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="G8" s="3">
-        <v>45155</v>
+        <v>45345</v>
       </c>
       <c r="H8" s="3">
-        <v>45250</v>
+        <v>45383</v>
       </c>
       <c r="I8" s="3">
-        <v>45279</v>
+        <v>45762</v>
       </c>
       <c r="J8" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="K8" t="s">
         <v>1</v>
       </c>
       <c r="L8" s="3">
-        <v>45152</v>
+        <v>45343</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
@@ -1400,37 +1382,37 @@
         <v>0</v>
       </c>
       <c r="B9" t="s">
-        <v>11</v>
+        <v>191</v>
       </c>
       <c r="C9" s="2">
         <v>1</v>
       </c>
       <c r="D9" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9" t="s">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="F9" t="s">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="G9" s="3">
-        <v>45345</v>
+        <v>45400</v>
       </c>
       <c r="H9" s="3">
-        <v>45383</v>
+        <v>45425</v>
       </c>
       <c r="I9" s="3">
-        <v>45762</v>
+        <v>45456</v>
       </c>
       <c r="J9" t="s">
-        <v>14</v>
+        <v>190</v>
       </c>
       <c r="K9" t="s">
         <v>1</v>
       </c>
       <c r="L9" s="3">
-        <v>45343</v>
+        <v>45400</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
@@ -1438,7 +1420,7 @@
         <v>0</v>
       </c>
       <c r="B10" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="C10" s="2">
         <v>1</v>
@@ -1447,28 +1429,28 @@
         <v>1</v>
       </c>
       <c r="E10" t="s">
-        <v>28</v>
+        <v>193</v>
       </c>
       <c r="F10" t="s">
-        <v>29</v>
+        <v>194</v>
       </c>
       <c r="G10" s="3">
-        <v>45400</v>
+        <v>45461</v>
       </c>
       <c r="H10" s="3">
-        <v>45425</v>
+        <v>45491</v>
       </c>
       <c r="I10" s="3">
-        <v>45456</v>
+        <v>45532</v>
       </c>
       <c r="J10" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="K10" t="s">
         <v>1</v>
       </c>
       <c r="L10" s="3">
-        <v>45400</v>
+        <v>45460</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
@@ -1476,37 +1458,37 @@
         <v>0</v>
       </c>
       <c r="B11" t="s">
-        <v>198</v>
+        <v>15</v>
       </c>
       <c r="C11" s="2">
         <v>1</v>
       </c>
       <c r="D11" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E11" t="s">
-        <v>199</v>
+        <v>16</v>
       </c>
       <c r="F11" t="s">
-        <v>200</v>
+        <v>17</v>
       </c>
       <c r="G11" s="3">
-        <v>45461</v>
+        <v>45509</v>
       </c>
       <c r="H11" s="3">
-        <v>45491</v>
+        <v>45678</v>
       </c>
       <c r="I11" s="3">
-        <v>45532</v>
+        <v>45800</v>
       </c>
       <c r="J11" t="s">
-        <v>196</v>
+        <v>14</v>
       </c>
       <c r="K11" t="s">
         <v>1</v>
       </c>
       <c r="L11" s="3">
-        <v>45460</v>
+        <v>45509</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
@@ -1514,7 +1496,7 @@
         <v>0</v>
       </c>
       <c r="B12" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C12" s="2">
         <v>1</v>
@@ -1523,19 +1505,19 @@
         <v>0</v>
       </c>
       <c r="E12" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F12" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="G12" s="3">
-        <v>45509</v>
+        <v>45534</v>
       </c>
       <c r="H12" s="3">
-        <v>45678</v>
+        <v>45580</v>
       </c>
       <c r="I12" s="3">
-        <v>45800</v>
+        <v>45874</v>
       </c>
       <c r="J12" t="s">
         <v>14</v>
@@ -1544,7 +1526,7 @@
         <v>1</v>
       </c>
       <c r="L12" s="3">
-        <v>45509</v>
+        <v>45532</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
@@ -1552,7 +1534,7 @@
         <v>0</v>
       </c>
       <c r="B13" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C13" s="2">
         <v>1</v>
@@ -1561,19 +1543,19 @@
         <v>0</v>
       </c>
       <c r="E13" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F13" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="G13" s="3">
-        <v>45519</v>
+        <v>45553</v>
       </c>
       <c r="H13" s="3">
-        <v>45623</v>
+        <v>45554</v>
       </c>
       <c r="I13" s="3">
-        <v>45888</v>
+        <v>45586</v>
       </c>
       <c r="J13" t="s">
         <v>2</v>
@@ -1582,7 +1564,7 @@
         <v>1</v>
       </c>
       <c r="L13" s="3">
-        <v>45510</v>
+        <v>45551</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
@@ -1590,7 +1572,7 @@
         <v>0</v>
       </c>
       <c r="B14" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C14" s="2">
         <v>1</v>
@@ -1599,19 +1581,19 @@
         <v>0</v>
       </c>
       <c r="E14" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F14" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="G14" s="3">
-        <v>45534</v>
+        <v>45569</v>
       </c>
       <c r="H14" s="3">
-        <v>45580</v>
+        <v>45694</v>
       </c>
       <c r="I14" s="3">
-        <v>45874</v>
+        <v>45903</v>
       </c>
       <c r="J14" t="s">
         <v>14</v>
@@ -1620,7 +1602,7 @@
         <v>1</v>
       </c>
       <c r="L14" s="3">
-        <v>45532</v>
+        <v>45565</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
@@ -1628,7 +1610,7 @@
         <v>0</v>
       </c>
       <c r="B15" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C15" s="2">
         <v>1</v>
@@ -1637,19 +1619,19 @@
         <v>0</v>
       </c>
       <c r="E15" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F15" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="G15" s="3">
-        <v>45553</v>
+        <v>45581</v>
       </c>
       <c r="H15" s="3">
-        <v>45554</v>
+        <v>45583</v>
       </c>
       <c r="I15" s="3">
-        <v>45586</v>
+        <v>45881</v>
       </c>
       <c r="J15" t="s">
         <v>2</v>
@@ -1658,7 +1640,7 @@
         <v>1</v>
       </c>
       <c r="L15" s="3">
-        <v>45551</v>
+        <v>45581</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
@@ -1666,7 +1648,7 @@
         <v>0</v>
       </c>
       <c r="B16" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C16" s="2">
         <v>1</v>
@@ -1675,28 +1657,28 @@
         <v>0</v>
       </c>
       <c r="E16" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F16" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="G16" s="3">
-        <v>45569</v>
+        <v>45588</v>
       </c>
       <c r="H16" s="3">
-        <v>45694</v>
+        <v>45593</v>
       </c>
       <c r="I16" s="3">
-        <v>45903</v>
+        <v>45888</v>
       </c>
       <c r="J16" t="s">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="K16" t="s">
         <v>1</v>
       </c>
       <c r="L16" s="3">
-        <v>45565</v>
+        <v>45588</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
@@ -1704,7 +1686,7 @@
         <v>0</v>
       </c>
       <c r="B17" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C17" s="2">
         <v>1</v>
@@ -1713,28 +1695,28 @@
         <v>0</v>
       </c>
       <c r="E17" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="F17" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="G17" s="3">
-        <v>45581</v>
+        <v>45593</v>
       </c>
       <c r="H17" s="3">
-        <v>45583</v>
+        <v>45629</v>
       </c>
       <c r="I17" s="3">
-        <v>45881</v>
+        <v>45894</v>
       </c>
       <c r="J17" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="K17" t="s">
         <v>1</v>
       </c>
       <c r="L17" s="3">
-        <v>45581</v>
+        <v>45589</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
@@ -1742,37 +1724,37 @@
         <v>0</v>
       </c>
       <c r="B18" t="s">
-        <v>33</v>
+        <v>195</v>
       </c>
       <c r="C18" s="2">
         <v>1</v>
       </c>
       <c r="D18" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E18" t="s">
-        <v>34</v>
+        <v>84</v>
       </c>
       <c r="F18" t="s">
-        <v>35</v>
+        <v>85</v>
       </c>
       <c r="G18" s="3">
-        <v>45588</v>
+        <v>45645</v>
       </c>
       <c r="H18" s="3">
-        <v>45593</v>
+        <v>45645</v>
       </c>
       <c r="I18" s="3">
-        <v>45888</v>
+        <v>45681</v>
       </c>
       <c r="J18" t="s">
-        <v>2</v>
+        <v>190</v>
       </c>
       <c r="K18" t="s">
         <v>1</v>
       </c>
       <c r="L18" s="3">
-        <v>45588</v>
+        <v>45645</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
@@ -1795,13 +1777,13 @@
         <v>38</v>
       </c>
       <c r="G19" s="3">
-        <v>45593</v>
+        <v>45681</v>
       </c>
       <c r="H19" s="3">
-        <v>45629</v>
+        <v>45769</v>
       </c>
       <c r="I19" s="3">
-        <v>45894</v>
+        <v>45912</v>
       </c>
       <c r="J19" t="s">
         <v>14</v>
@@ -1810,7 +1792,7 @@
         <v>1</v>
       </c>
       <c r="L19" s="3">
-        <v>45589</v>
+        <v>45679</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
@@ -1818,37 +1800,37 @@
         <v>0</v>
       </c>
       <c r="B20" t="s">
-        <v>201</v>
+        <v>39</v>
       </c>
       <c r="C20" s="2">
         <v>1</v>
       </c>
       <c r="D20" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E20" t="s">
-        <v>87</v>
+        <v>40</v>
       </c>
       <c r="F20" t="s">
-        <v>88</v>
+        <v>41</v>
       </c>
       <c r="G20" s="3">
-        <v>45645</v>
+        <v>45700</v>
       </c>
       <c r="H20" s="3">
-        <v>45645</v>
+        <v>45740</v>
       </c>
       <c r="I20" s="3">
-        <v>45681</v>
+        <v>45896</v>
       </c>
       <c r="J20" t="s">
-        <v>196</v>
+        <v>14</v>
       </c>
       <c r="K20" t="s">
         <v>1</v>
       </c>
       <c r="L20" s="3">
-        <v>45645</v>
+        <v>45698</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
@@ -1856,7 +1838,7 @@
         <v>0</v>
       </c>
       <c r="B21" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C21" s="2">
         <v>1</v>
@@ -1865,19 +1847,19 @@
         <v>0</v>
       </c>
       <c r="E21" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="F21" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="G21" s="3">
-        <v>45681</v>
+        <v>45700</v>
       </c>
       <c r="H21" s="3">
-        <v>45769</v>
+        <v>45741</v>
       </c>
       <c r="I21" s="3">
-        <v>45912</v>
+        <v>45868</v>
       </c>
       <c r="J21" t="s">
         <v>14</v>
@@ -1886,7 +1868,7 @@
         <v>1</v>
       </c>
       <c r="L21" s="3">
-        <v>45679</v>
+        <v>45698</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
@@ -1894,7 +1876,7 @@
         <v>0</v>
       </c>
       <c r="B22" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C22" s="2">
         <v>1</v>
@@ -1903,19 +1885,19 @@
         <v>0</v>
       </c>
       <c r="E22" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="F22" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="G22" s="3">
-        <v>45700</v>
+        <v>45755</v>
       </c>
       <c r="H22" s="3">
-        <v>45740</v>
+        <v>45898</v>
       </c>
       <c r="I22" s="3">
-        <v>45896</v>
+        <v>45987</v>
       </c>
       <c r="J22" t="s">
         <v>14</v>
@@ -1924,7 +1906,7 @@
         <v>1</v>
       </c>
       <c r="L22" s="3">
-        <v>45698</v>
+        <v>45748</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
@@ -1932,7 +1914,7 @@
         <v>0</v>
       </c>
       <c r="B23" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C23" s="2">
         <v>1</v>
@@ -1941,28 +1923,28 @@
         <v>0</v>
       </c>
       <c r="E23" t="s">
-        <v>46</v>
+        <v>12</v>
       </c>
       <c r="F23" t="s">
-        <v>47</v>
+        <v>13</v>
       </c>
       <c r="G23" s="3">
-        <v>45700</v>
+        <v>45762</v>
       </c>
       <c r="H23" s="3">
-        <v>45741</v>
+        <v>45796</v>
       </c>
       <c r="I23" s="3">
-        <v>45868</v>
+        <v>45947</v>
       </c>
       <c r="J23" t="s">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="K23" t="s">
         <v>1</v>
       </c>
       <c r="L23" s="3">
-        <v>45698</v>
+        <v>45761</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
@@ -1970,7 +1952,7 @@
         <v>0</v>
       </c>
       <c r="B24" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C24" s="2">
         <v>1</v>
@@ -1979,28 +1961,28 @@
         <v>0</v>
       </c>
       <c r="E24" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F24" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G24" s="3">
-        <v>45755</v>
+        <v>45762</v>
       </c>
       <c r="H24" s="3">
-        <v>45898</v>
+        <v>45863</v>
       </c>
       <c r="I24" s="3">
-        <v>45987</v>
+        <v>45910</v>
       </c>
       <c r="J24" t="s">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="K24" t="s">
         <v>1</v>
       </c>
       <c r="L24" s="3">
-        <v>45748</v>
+        <v>45761</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
@@ -2008,7 +1990,7 @@
         <v>0</v>
       </c>
       <c r="B25" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C25" s="2">
         <v>1</v>
@@ -2017,19 +1999,19 @@
         <v>0</v>
       </c>
       <c r="E25" t="s">
-        <v>12</v>
+        <v>53</v>
       </c>
       <c r="F25" t="s">
-        <v>13</v>
+        <v>54</v>
       </c>
       <c r="G25" s="3">
-        <v>45762</v>
+        <v>45779</v>
       </c>
       <c r="H25" s="3">
-        <v>45796</v>
+        <v>45880</v>
       </c>
       <c r="I25" s="3">
-        <v>45947</v>
+        <v>45916</v>
       </c>
       <c r="J25" t="s">
         <v>2</v>
@@ -2038,7 +2020,7 @@
         <v>1</v>
       </c>
       <c r="L25" s="3">
-        <v>45761</v>
+        <v>45777</v>
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.25">
@@ -2046,7 +2028,7 @@
         <v>0</v>
       </c>
       <c r="B26" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C26" s="2">
         <v>1</v>
@@ -2061,13 +2043,13 @@
         <v>54</v>
       </c>
       <c r="G26" s="3">
-        <v>45762</v>
+        <v>45779</v>
       </c>
       <c r="H26" s="3">
-        <v>45863</v>
+        <v>45880</v>
       </c>
       <c r="I26" s="3">
-        <v>45910</v>
+        <v>45916</v>
       </c>
       <c r="J26" t="s">
         <v>2</v>
@@ -2076,7 +2058,7 @@
         <v>1</v>
       </c>
       <c r="L26" s="3">
-        <v>45761</v>
+        <v>45777</v>
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.25">
@@ -2084,7 +2066,7 @@
         <v>0</v>
       </c>
       <c r="B27" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C27" s="2">
         <v>1</v>
@@ -2093,19 +2075,19 @@
         <v>0</v>
       </c>
       <c r="E27" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F27" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G27" s="3">
-        <v>45779</v>
+        <v>45786</v>
       </c>
       <c r="H27" s="3">
-        <v>45880</v>
+        <v>45800</v>
       </c>
       <c r="I27" s="3">
-        <v>45916</v>
+        <v>45915</v>
       </c>
       <c r="J27" t="s">
         <v>2</v>
@@ -2114,7 +2096,7 @@
         <v>1</v>
       </c>
       <c r="L27" s="3">
-        <v>45777</v>
+        <v>45782</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
@@ -2122,7 +2104,7 @@
         <v>0</v>
       </c>
       <c r="B28" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C28" s="2">
         <v>1</v>
@@ -2131,19 +2113,19 @@
         <v>0</v>
       </c>
       <c r="E28" t="s">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="F28" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="G28" s="3">
-        <v>45779</v>
+        <v>45784</v>
       </c>
       <c r="H28" s="3">
-        <v>45880</v>
+        <v>45827</v>
       </c>
       <c r="I28" s="3">
-        <v>45916</v>
+        <v>45895</v>
       </c>
       <c r="J28" t="s">
         <v>2</v>
@@ -2152,7 +2134,7 @@
         <v>1</v>
       </c>
       <c r="L28" s="3">
-        <v>45777</v>
+        <v>45782</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
@@ -2160,7 +2142,7 @@
         <v>0</v>
       </c>
       <c r="B29" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C29" s="2">
         <v>1</v>
@@ -2169,19 +2151,19 @@
         <v>0</v>
       </c>
       <c r="E29" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F29" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G29" s="3">
-        <v>45786</v>
+        <v>45793</v>
       </c>
       <c r="H29" s="3">
-        <v>45800</v>
+        <v>45827</v>
       </c>
       <c r="I29" s="3">
-        <v>45915</v>
+        <v>45908</v>
       </c>
       <c r="J29" t="s">
         <v>2</v>
@@ -2190,7 +2172,7 @@
         <v>1</v>
       </c>
       <c r="L29" s="3">
-        <v>45782</v>
+        <v>45789</v>
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
@@ -2198,7 +2180,7 @@
         <v>0</v>
       </c>
       <c r="B30" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C30" s="2">
         <v>1</v>
@@ -2207,28 +2189,28 @@
         <v>0</v>
       </c>
       <c r="E30" t="s">
-        <v>37</v>
+        <v>64</v>
       </c>
       <c r="F30" t="s">
-        <v>38</v>
+        <v>65</v>
       </c>
       <c r="G30" s="3">
-        <v>45784</v>
+        <v>45796</v>
       </c>
       <c r="H30" s="3">
-        <v>45827</v>
+        <v>45821</v>
       </c>
       <c r="I30" s="3">
-        <v>45895</v>
+        <v>45931</v>
       </c>
       <c r="J30" t="s">
-        <v>2</v>
+        <v>66</v>
       </c>
       <c r="K30" t="s">
         <v>1</v>
       </c>
       <c r="L30" s="3">
-        <v>45782</v>
+        <v>45796</v>
       </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
@@ -2236,7 +2218,7 @@
         <v>0</v>
       </c>
       <c r="B31" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C31" s="2">
         <v>1</v>
@@ -2245,19 +2227,19 @@
         <v>0</v>
       </c>
       <c r="E31" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="F31" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="G31" s="3">
-        <v>45793</v>
+        <v>45798</v>
       </c>
       <c r="H31" s="3">
-        <v>45827</v>
+        <v>45799</v>
       </c>
       <c r="I31" s="3">
-        <v>45908</v>
+        <v>45909</v>
       </c>
       <c r="J31" t="s">
         <v>2</v>
@@ -2266,7 +2248,7 @@
         <v>1</v>
       </c>
       <c r="L31" s="3">
-        <v>45789</v>
+        <v>45797</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.25">
@@ -2274,7 +2256,7 @@
         <v>0</v>
       </c>
       <c r="B32" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C32" s="2">
         <v>1</v>
@@ -2283,28 +2265,28 @@
         <v>0</v>
       </c>
       <c r="E32" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="F32" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="G32" s="3">
-        <v>45796</v>
+        <v>45799</v>
       </c>
       <c r="H32" s="3">
-        <v>45821</v>
+        <v>45817</v>
       </c>
       <c r="I32" s="3">
-        <v>45931</v>
+        <v>45924</v>
       </c>
       <c r="J32" t="s">
-        <v>69</v>
+        <v>14</v>
       </c>
       <c r="K32" t="s">
         <v>1</v>
       </c>
       <c r="L32" s="3">
-        <v>45796</v>
+        <v>45799</v>
       </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.25">
@@ -2312,7 +2294,7 @@
         <v>0</v>
       </c>
       <c r="B33" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C33" s="2">
         <v>1</v>
@@ -2321,19 +2303,19 @@
         <v>0</v>
       </c>
       <c r="E33" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="F33" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="G33" s="3">
-        <v>45798</v>
+        <v>45800</v>
       </c>
       <c r="H33" s="3">
-        <v>45799</v>
+        <v>45812</v>
       </c>
       <c r="I33" s="3">
-        <v>45909</v>
+        <v>45896</v>
       </c>
       <c r="J33" t="s">
         <v>2</v>
@@ -2342,7 +2324,7 @@
         <v>1</v>
       </c>
       <c r="L33" s="3">
-        <v>45797</v>
+        <v>45800</v>
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.25">
@@ -2350,7 +2332,7 @@
         <v>0</v>
       </c>
       <c r="B34" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C34" s="2">
         <v>1</v>
@@ -2359,19 +2341,19 @@
         <v>0</v>
       </c>
       <c r="E34" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="F34" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="G34" s="3">
-        <v>45799</v>
+        <v>45804</v>
       </c>
       <c r="H34" s="3">
-        <v>45817</v>
+        <v>45923</v>
       </c>
       <c r="I34" s="3">
-        <v>45924</v>
+        <v>46013</v>
       </c>
       <c r="J34" t="s">
         <v>14</v>
@@ -2380,7 +2362,7 @@
         <v>1</v>
       </c>
       <c r="L34" s="3">
-        <v>45799</v>
+        <v>45804</v>
       </c>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.25">
@@ -2388,7 +2370,7 @@
         <v>0</v>
       </c>
       <c r="B35" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="C35" s="2">
         <v>1</v>
@@ -2397,19 +2379,19 @@
         <v>0</v>
       </c>
       <c r="E35" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="F35" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="G35" s="3">
-        <v>45800</v>
+        <v>45810</v>
       </c>
       <c r="H35" s="3">
-        <v>45812</v>
+        <v>45848</v>
       </c>
       <c r="I35" s="3">
-        <v>45896</v>
+        <v>45912</v>
       </c>
       <c r="J35" t="s">
         <v>2</v>
@@ -2418,7 +2400,7 @@
         <v>1</v>
       </c>
       <c r="L35" s="3">
-        <v>45800</v>
+        <v>45806</v>
       </c>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.25">
@@ -2426,7 +2408,7 @@
         <v>0</v>
       </c>
       <c r="B36" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C36" s="2">
         <v>1</v>
@@ -2435,28 +2417,28 @@
         <v>0</v>
       </c>
       <c r="E36" t="s">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="F36" t="s">
-        <v>81</v>
+        <v>51</v>
       </c>
       <c r="G36" s="3">
-        <v>45804</v>
+        <v>45810</v>
       </c>
       <c r="H36" s="3">
-        <v>45923</v>
+        <v>45853</v>
       </c>
       <c r="I36" s="3">
-        <v>46013</v>
+        <v>45915</v>
       </c>
       <c r="J36" t="s">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="K36" t="s">
         <v>1</v>
       </c>
       <c r="L36" s="3">
-        <v>45804</v>
+        <v>45806</v>
       </c>
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.25">
@@ -2464,7 +2446,7 @@
         <v>0</v>
       </c>
       <c r="B37" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C37" s="2">
         <v>1</v>
@@ -2473,28 +2455,28 @@
         <v>0</v>
       </c>
       <c r="E37" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F37" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="G37" s="3">
-        <v>45810</v>
+        <v>45811</v>
       </c>
       <c r="H37" s="3">
-        <v>45848</v>
+        <v>45979</v>
       </c>
       <c r="I37" s="3">
-        <v>45912</v>
+        <v>46014</v>
       </c>
       <c r="J37" t="s">
-        <v>2</v>
+        <v>86</v>
       </c>
       <c r="K37" t="s">
         <v>1</v>
       </c>
       <c r="L37" s="3">
-        <v>45806</v>
+        <v>45811</v>
       </c>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.25">
@@ -2502,7 +2484,7 @@
         <v>0</v>
       </c>
       <c r="B38" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C38" s="2">
         <v>1</v>
@@ -2511,19 +2493,19 @@
         <v>0</v>
       </c>
       <c r="E38" t="s">
-        <v>53</v>
+        <v>88</v>
       </c>
       <c r="F38" t="s">
-        <v>54</v>
+        <v>89</v>
       </c>
       <c r="G38" s="3">
-        <v>45810</v>
+        <v>45811</v>
       </c>
       <c r="H38" s="3">
-        <v>45853</v>
+        <v>45821</v>
       </c>
       <c r="I38" s="3">
-        <v>45915</v>
+        <v>45910</v>
       </c>
       <c r="J38" t="s">
         <v>2</v>
@@ -2532,7 +2514,7 @@
         <v>1</v>
       </c>
       <c r="L38" s="3">
-        <v>45806</v>
+        <v>45811</v>
       </c>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.25">
@@ -2540,7 +2522,7 @@
         <v>0</v>
       </c>
       <c r="B39" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C39" s="2">
         <v>1</v>
@@ -2549,22 +2531,22 @@
         <v>0</v>
       </c>
       <c r="E39" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="F39" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="G39" s="3">
         <v>45811</v>
       </c>
       <c r="H39" s="3">
-        <v>45979</v>
+        <v>45820</v>
       </c>
       <c r="I39" s="3">
-        <v>46014</v>
+        <v>45978</v>
       </c>
       <c r="J39" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="K39" t="s">
         <v>1</v>
@@ -2578,7 +2560,7 @@
         <v>0</v>
       </c>
       <c r="B40" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C40" s="2">
         <v>1</v>
@@ -2587,19 +2569,19 @@
         <v>0</v>
       </c>
       <c r="E40" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="F40" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="G40" s="3">
         <v>45811</v>
       </c>
       <c r="H40" s="3">
-        <v>45821</v>
+        <v>45812</v>
       </c>
       <c r="I40" s="3">
-        <v>45910</v>
+        <v>45926</v>
       </c>
       <c r="J40" t="s">
         <v>2</v>
@@ -2616,7 +2598,7 @@
         <v>0</v>
       </c>
       <c r="B41" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C41" s="2">
         <v>1</v>
@@ -2625,22 +2607,22 @@
         <v>0</v>
       </c>
       <c r="E41" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="F41" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="G41" s="3">
         <v>45811</v>
       </c>
       <c r="H41" s="3">
-        <v>45820</v>
+        <v>45860</v>
       </c>
       <c r="I41" s="3">
-        <v>45978</v>
+        <v>45904</v>
       </c>
       <c r="J41" t="s">
-        <v>96</v>
+        <v>2</v>
       </c>
       <c r="K41" t="s">
         <v>1</v>
@@ -2654,7 +2636,7 @@
         <v>0</v>
       </c>
       <c r="B42" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="C42" s="2">
         <v>1</v>
@@ -2663,19 +2645,19 @@
         <v>0</v>
       </c>
       <c r="E42" t="s">
-        <v>98</v>
+        <v>25</v>
       </c>
       <c r="F42" t="s">
-        <v>99</v>
+        <v>26</v>
       </c>
       <c r="G42" s="3">
-        <v>45811</v>
+        <v>45813</v>
       </c>
       <c r="H42" s="3">
-        <v>45812</v>
+        <v>45814</v>
       </c>
       <c r="I42" s="3">
-        <v>45926</v>
+        <v>45896</v>
       </c>
       <c r="J42" t="s">
         <v>2</v>
@@ -2684,7 +2666,7 @@
         <v>1</v>
       </c>
       <c r="L42" s="3">
-        <v>45811</v>
+        <v>45812</v>
       </c>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.25">
@@ -2692,7 +2674,7 @@
         <v>0</v>
       </c>
       <c r="B43" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C43" s="2">
         <v>1</v>
@@ -2701,19 +2683,19 @@
         <v>0</v>
       </c>
       <c r="E43" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F43" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G43" s="3">
-        <v>45811</v>
+        <v>45813</v>
       </c>
       <c r="H43" s="3">
-        <v>45860</v>
+        <v>45827</v>
       </c>
       <c r="I43" s="3">
-        <v>45904</v>
+        <v>45897</v>
       </c>
       <c r="J43" t="s">
         <v>2</v>
@@ -2722,7 +2704,7 @@
         <v>1</v>
       </c>
       <c r="L43" s="3">
-        <v>45811</v>
+        <v>45812</v>
       </c>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.25">
@@ -2730,7 +2712,7 @@
         <v>0</v>
       </c>
       <c r="B44" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C44" s="2">
         <v>1</v>
@@ -2739,19 +2721,19 @@
         <v>0</v>
       </c>
       <c r="E44" t="s">
-        <v>28</v>
+        <v>105</v>
       </c>
       <c r="F44" t="s">
-        <v>29</v>
+        <v>106</v>
       </c>
       <c r="G44" s="3">
-        <v>45813</v>
+        <v>45824</v>
       </c>
       <c r="H44" s="3">
-        <v>45814</v>
+        <v>45912</v>
       </c>
       <c r="I44" s="3">
-        <v>45896</v>
+        <v>45994</v>
       </c>
       <c r="J44" t="s">
         <v>2</v>
@@ -2760,7 +2742,7 @@
         <v>1</v>
       </c>
       <c r="L44" s="3">
-        <v>45812</v>
+        <v>45824</v>
       </c>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.25">
@@ -2768,7 +2750,7 @@
         <v>0</v>
       </c>
       <c r="B45" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C45" s="2">
         <v>1</v>
@@ -2777,19 +2759,19 @@
         <v>0</v>
       </c>
       <c r="E45" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="F45" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="G45" s="3">
-        <v>45813</v>
+        <v>45833</v>
       </c>
       <c r="H45" s="3">
-        <v>45827</v>
+        <v>45839</v>
       </c>
       <c r="I45" s="3">
-        <v>45897</v>
+        <v>45908</v>
       </c>
       <c r="J45" t="s">
         <v>2</v>
@@ -2798,7 +2780,7 @@
         <v>1</v>
       </c>
       <c r="L45" s="3">
-        <v>45812</v>
+        <v>45833</v>
       </c>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.25">
@@ -2806,7 +2788,7 @@
         <v>0</v>
       </c>
       <c r="B46" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C46" s="2">
         <v>1</v>
@@ -2821,13 +2803,13 @@
         <v>109</v>
       </c>
       <c r="G46" s="3">
-        <v>45824</v>
+        <v>45833</v>
       </c>
       <c r="H46" s="3">
-        <v>45912</v>
+        <v>45839</v>
       </c>
       <c r="I46" s="3">
-        <v>45994</v>
+        <v>45911</v>
       </c>
       <c r="J46" t="s">
         <v>2</v>
@@ -2836,7 +2818,7 @@
         <v>1</v>
       </c>
       <c r="L46" s="3">
-        <v>45824</v>
+        <v>45833</v>
       </c>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.25">
@@ -2844,7 +2826,7 @@
         <v>0</v>
       </c>
       <c r="B47" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C47" s="2">
         <v>1</v>
@@ -2853,19 +2835,19 @@
         <v>0</v>
       </c>
       <c r="E47" t="s">
-        <v>111</v>
+        <v>88</v>
       </c>
       <c r="F47" t="s">
-        <v>112</v>
+        <v>89</v>
       </c>
       <c r="G47" s="3">
-        <v>45833</v>
+        <v>45834</v>
       </c>
       <c r="H47" s="3">
-        <v>45839</v>
+        <v>45884</v>
       </c>
       <c r="I47" s="3">
-        <v>45908</v>
+        <v>45950</v>
       </c>
       <c r="J47" t="s">
         <v>2</v>
@@ -2874,7 +2856,7 @@
         <v>1</v>
       </c>
       <c r="L47" s="3">
-        <v>45833</v>
+        <v>45834</v>
       </c>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.25">
@@ -2882,37 +2864,37 @@
         <v>0</v>
       </c>
       <c r="B48" t="s">
+        <v>112</v>
+      </c>
+      <c r="C48" s="2">
+        <v>1</v>
+      </c>
+      <c r="D48" s="2">
+        <v>0</v>
+      </c>
+      <c r="E48" t="s">
         <v>113</v>
       </c>
-      <c r="C48" s="2">
-        <v>1</v>
-      </c>
-      <c r="D48" s="2">
-        <v>0</v>
-      </c>
-      <c r="E48" t="s">
-        <v>111</v>
-      </c>
       <c r="F48" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G48" s="3">
-        <v>45833</v>
+        <v>45834</v>
       </c>
       <c r="H48" s="3">
-        <v>45839</v>
+        <v>45849</v>
       </c>
       <c r="I48" s="3">
-        <v>45911</v>
+        <v>45947</v>
       </c>
       <c r="J48" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="K48" t="s">
         <v>1</v>
       </c>
       <c r="L48" s="3">
-        <v>45833</v>
+        <v>45834</v>
       </c>
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.25">
@@ -2920,28 +2902,28 @@
         <v>0</v>
       </c>
       <c r="B49" t="s">
+        <v>115</v>
+      </c>
+      <c r="C49" s="2">
+        <v>1</v>
+      </c>
+      <c r="D49" s="2">
+        <v>0</v>
+      </c>
+      <c r="E49" t="s">
+        <v>113</v>
+      </c>
+      <c r="F49" t="s">
         <v>114</v>
-      </c>
-      <c r="C49" s="2">
-        <v>1</v>
-      </c>
-      <c r="D49" s="2">
-        <v>0</v>
-      </c>
-      <c r="E49" t="s">
-        <v>91</v>
-      </c>
-      <c r="F49" t="s">
-        <v>92</v>
       </c>
       <c r="G49" s="3">
         <v>45834</v>
       </c>
       <c r="H49" s="3">
-        <v>45884</v>
+        <v>45905</v>
       </c>
       <c r="I49" s="3">
-        <v>45950</v>
+        <v>45972</v>
       </c>
       <c r="J49" t="s">
         <v>2</v>
@@ -2958,7 +2940,7 @@
         <v>0</v>
       </c>
       <c r="B50" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C50" s="2">
         <v>1</v>
@@ -2967,28 +2949,28 @@
         <v>0</v>
       </c>
       <c r="E50" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F50" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G50" s="3">
-        <v>45834</v>
+        <v>45835</v>
       </c>
       <c r="H50" s="3">
-        <v>45849</v>
+        <v>45853</v>
       </c>
       <c r="I50" s="3">
-        <v>45947</v>
+        <v>45901</v>
       </c>
       <c r="J50" t="s">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="K50" t="s">
         <v>1</v>
       </c>
       <c r="L50" s="3">
-        <v>45834</v>
+        <v>45835</v>
       </c>
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.25">
@@ -2996,37 +2978,37 @@
         <v>0</v>
       </c>
       <c r="B51" t="s">
+        <v>119</v>
+      </c>
+      <c r="C51" s="2">
+        <v>1</v>
+      </c>
+      <c r="D51" s="2">
+        <v>0</v>
+      </c>
+      <c r="E51" t="s">
+        <v>117</v>
+      </c>
+      <c r="F51" t="s">
         <v>118</v>
       </c>
-      <c r="C51" s="2">
-        <v>1</v>
-      </c>
-      <c r="D51" s="2">
-        <v>0</v>
-      </c>
-      <c r="E51" t="s">
-        <v>116</v>
-      </c>
-      <c r="F51" t="s">
-        <v>117</v>
-      </c>
       <c r="G51" s="3">
-        <v>45834</v>
+        <v>45835</v>
       </c>
       <c r="H51" s="3">
-        <v>45905</v>
+        <v>45933</v>
       </c>
       <c r="I51" s="3">
         <v>45972</v>
       </c>
       <c r="J51" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="K51" t="s">
         <v>1</v>
       </c>
       <c r="L51" s="3">
-        <v>45834</v>
+        <v>45835</v>
       </c>
     </row>
     <row r="52" spans="1:12" x14ac:dyDescent="0.25">
@@ -3034,7 +3016,7 @@
         <v>0</v>
       </c>
       <c r="B52" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C52" s="2">
         <v>1</v>
@@ -3043,22 +3025,22 @@
         <v>0</v>
       </c>
       <c r="E52" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="F52" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="G52" s="3">
         <v>45835</v>
       </c>
       <c r="H52" s="3">
-        <v>45853</v>
+        <v>45933</v>
       </c>
       <c r="I52" s="3">
-        <v>45901</v>
+        <v>45972</v>
       </c>
       <c r="J52" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="K52" t="s">
         <v>1</v>
@@ -3072,7 +3054,7 @@
         <v>0</v>
       </c>
       <c r="B53" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C53" s="2">
         <v>1</v>
@@ -3081,22 +3063,22 @@
         <v>0</v>
       </c>
       <c r="E53" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="F53" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="G53" s="3">
         <v>45835</v>
       </c>
       <c r="H53" s="3">
-        <v>45933</v>
+        <v>45847</v>
       </c>
       <c r="I53" s="3">
-        <v>45972</v>
+        <v>45901</v>
       </c>
       <c r="J53" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="K53" t="s">
         <v>1</v>
@@ -3110,7 +3092,7 @@
         <v>0</v>
       </c>
       <c r="B54" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C54" s="2">
         <v>1</v>
@@ -3119,28 +3101,28 @@
         <v>0</v>
       </c>
       <c r="E54" t="s">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="F54" t="s">
-        <v>121</v>
+        <v>51</v>
       </c>
       <c r="G54" s="3">
-        <v>45835</v>
+        <v>45839</v>
       </c>
       <c r="H54" s="3">
         <v>45933</v>
       </c>
       <c r="I54" s="3">
-        <v>45972</v>
+        <v>45959</v>
       </c>
       <c r="J54" t="s">
-        <v>6</v>
+        <v>86</v>
       </c>
       <c r="K54" t="s">
         <v>1</v>
       </c>
       <c r="L54" s="3">
-        <v>45835</v>
+        <v>45839</v>
       </c>
     </row>
     <row r="55" spans="1:12" x14ac:dyDescent="0.25">
@@ -3148,7 +3130,7 @@
         <v>0</v>
       </c>
       <c r="B55" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C55" s="2">
         <v>1</v>
@@ -3157,19 +3139,19 @@
         <v>0</v>
       </c>
       <c r="E55" t="s">
-        <v>120</v>
+        <v>31</v>
       </c>
       <c r="F55" t="s">
-        <v>121</v>
+        <v>32</v>
       </c>
       <c r="G55" s="3">
-        <v>45835</v>
+        <v>45846</v>
       </c>
       <c r="H55" s="3">
-        <v>45847</v>
+        <v>45854</v>
       </c>
       <c r="I55" s="3">
-        <v>45901</v>
+        <v>45888</v>
       </c>
       <c r="J55" t="s">
         <v>2</v>
@@ -3178,7 +3160,7 @@
         <v>1</v>
       </c>
       <c r="L55" s="3">
-        <v>45835</v>
+        <v>45846</v>
       </c>
     </row>
     <row r="56" spans="1:12" x14ac:dyDescent="0.25">
@@ -3186,7 +3168,7 @@
         <v>0</v>
       </c>
       <c r="B56" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C56" s="2">
         <v>1</v>
@@ -3195,28 +3177,28 @@
         <v>0</v>
       </c>
       <c r="E56" t="s">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="F56" t="s">
-        <v>54</v>
+        <v>35</v>
       </c>
       <c r="G56" s="3">
-        <v>45839</v>
+        <v>45847</v>
       </c>
       <c r="H56" s="3">
-        <v>45933</v>
+        <v>45860</v>
       </c>
       <c r="I56" s="3">
-        <v>45959</v>
+        <v>45897</v>
       </c>
       <c r="J56" t="s">
-        <v>89</v>
+        <v>2</v>
       </c>
       <c r="K56" t="s">
         <v>1</v>
       </c>
       <c r="L56" s="3">
-        <v>45839</v>
+        <v>45847</v>
       </c>
     </row>
     <row r="57" spans="1:12" x14ac:dyDescent="0.25">
@@ -3224,7 +3206,7 @@
         <v>0</v>
       </c>
       <c r="B57" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C57" s="2">
         <v>1</v>
@@ -3239,13 +3221,13 @@
         <v>35</v>
       </c>
       <c r="G57" s="3">
-        <v>45846</v>
+        <v>45847</v>
       </c>
       <c r="H57" s="3">
-        <v>45854</v>
+        <v>45849</v>
       </c>
       <c r="I57" s="3">
-        <v>45888</v>
+        <v>45894</v>
       </c>
       <c r="J57" t="s">
         <v>2</v>
@@ -3254,7 +3236,7 @@
         <v>1</v>
       </c>
       <c r="L57" s="3">
-        <v>45846</v>
+        <v>45847</v>
       </c>
     </row>
     <row r="58" spans="1:12" x14ac:dyDescent="0.25">
@@ -3262,28 +3244,28 @@
         <v>0</v>
       </c>
       <c r="B58" t="s">
+        <v>126</v>
+      </c>
+      <c r="C58" s="2">
+        <v>1</v>
+      </c>
+      <c r="D58" s="2">
+        <v>0</v>
+      </c>
+      <c r="E58" t="s">
         <v>127</v>
       </c>
-      <c r="C58" s="2">
-        <v>1</v>
-      </c>
-      <c r="D58" s="2">
-        <v>0</v>
-      </c>
-      <c r="E58" t="s">
-        <v>37</v>
-      </c>
       <c r="F58" t="s">
-        <v>38</v>
+        <v>128</v>
       </c>
       <c r="G58" s="3">
         <v>45847</v>
       </c>
       <c r="H58" s="3">
-        <v>45860</v>
+        <v>45852</v>
       </c>
       <c r="I58" s="3">
-        <v>45897</v>
+        <v>45894</v>
       </c>
       <c r="J58" t="s">
         <v>2</v>
@@ -3300,28 +3282,28 @@
         <v>0</v>
       </c>
       <c r="B59" t="s">
+        <v>129</v>
+      </c>
+      <c r="C59" s="2">
+        <v>1</v>
+      </c>
+      <c r="D59" s="2">
+        <v>0</v>
+      </c>
+      <c r="E59" t="s">
+        <v>127</v>
+      </c>
+      <c r="F59" t="s">
         <v>128</v>
-      </c>
-      <c r="C59" s="2">
-        <v>1</v>
-      </c>
-      <c r="D59" s="2">
-        <v>0</v>
-      </c>
-      <c r="E59" t="s">
-        <v>37</v>
-      </c>
-      <c r="F59" t="s">
-        <v>38</v>
       </c>
       <c r="G59" s="3">
         <v>45847</v>
       </c>
       <c r="H59" s="3">
-        <v>45849</v>
+        <v>45860</v>
       </c>
       <c r="I59" s="3">
-        <v>45894</v>
+        <v>45897</v>
       </c>
       <c r="J59" t="s">
         <v>2</v>
@@ -3338,7 +3320,7 @@
         <v>0</v>
       </c>
       <c r="B60" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C60" s="2">
         <v>1</v>
@@ -3347,19 +3329,19 @@
         <v>0</v>
       </c>
       <c r="E60" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F60" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G60" s="3">
         <v>45847</v>
       </c>
       <c r="H60" s="3">
-        <v>45852</v>
+        <v>45854</v>
       </c>
       <c r="I60" s="3">
-        <v>45894</v>
+        <v>45888</v>
       </c>
       <c r="J60" t="s">
         <v>2</v>
@@ -3376,28 +3358,28 @@
         <v>0</v>
       </c>
       <c r="B61" t="s">
+        <v>133</v>
+      </c>
+      <c r="C61" s="2">
+        <v>1</v>
+      </c>
+      <c r="D61" s="2">
+        <v>0</v>
+      </c>
+      <c r="E61" t="s">
+        <v>131</v>
+      </c>
+      <c r="F61" t="s">
         <v>132</v>
-      </c>
-      <c r="C61" s="2">
-        <v>1</v>
-      </c>
-      <c r="D61" s="2">
-        <v>0</v>
-      </c>
-      <c r="E61" t="s">
-        <v>130</v>
-      </c>
-      <c r="F61" t="s">
-        <v>131</v>
       </c>
       <c r="G61" s="3">
         <v>45847</v>
       </c>
       <c r="H61" s="3">
-        <v>45860</v>
+        <v>45854</v>
       </c>
       <c r="I61" s="3">
-        <v>45897</v>
+        <v>45894</v>
       </c>
       <c r="J61" t="s">
         <v>2</v>
@@ -3414,7 +3396,7 @@
         <v>0</v>
       </c>
       <c r="B62" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C62" s="2">
         <v>1</v>
@@ -3423,28 +3405,28 @@
         <v>0</v>
       </c>
       <c r="E62" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F62" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G62" s="3">
-        <v>45847</v>
+        <v>45848</v>
       </c>
       <c r="H62" s="3">
-        <v>45854</v>
+        <v>46016</v>
       </c>
       <c r="I62" s="3">
-        <v>45888</v>
+        <v>46107</v>
       </c>
       <c r="J62" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="K62" t="s">
         <v>1</v>
       </c>
       <c r="L62" s="3">
-        <v>45847</v>
+        <v>45848</v>
       </c>
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.25">
@@ -3452,7 +3434,7 @@
         <v>0</v>
       </c>
       <c r="B63" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C63" s="2">
         <v>1</v>
@@ -3461,19 +3443,19 @@
         <v>0</v>
       </c>
       <c r="E63" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="F63" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="G63" s="3">
-        <v>45847</v>
+        <v>45849</v>
       </c>
       <c r="H63" s="3">
-        <v>45854</v>
+        <v>45882</v>
       </c>
       <c r="I63" s="3">
-        <v>45894</v>
+        <v>45916</v>
       </c>
       <c r="J63" t="s">
         <v>2</v>
@@ -3482,7 +3464,7 @@
         <v>1</v>
       </c>
       <c r="L63" s="3">
-        <v>45847</v>
+        <v>45849</v>
       </c>
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.25">
@@ -3490,7 +3472,7 @@
         <v>0</v>
       </c>
       <c r="B64" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="C64" s="2">
         <v>1</v>
@@ -3505,22 +3487,22 @@
         <v>139</v>
       </c>
       <c r="G64" s="3">
-        <v>45848</v>
+        <v>45849</v>
       </c>
       <c r="H64" s="3">
-        <v>46016</v>
+        <v>45880</v>
       </c>
       <c r="I64" s="3">
-        <v>46107</v>
+        <v>45910</v>
       </c>
       <c r="J64" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="K64" t="s">
         <v>1</v>
       </c>
       <c r="L64" s="3">
-        <v>45848</v>
+        <v>45849</v>
       </c>
     </row>
     <row r="65" spans="1:12" x14ac:dyDescent="0.25">
@@ -3528,7 +3510,7 @@
         <v>0</v>
       </c>
       <c r="B65" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C65" s="2">
         <v>1</v>
@@ -3537,19 +3519,19 @@
         <v>0</v>
       </c>
       <c r="E65" t="s">
-        <v>141</v>
+        <v>117</v>
       </c>
       <c r="F65" t="s">
-        <v>142</v>
+        <v>118</v>
       </c>
       <c r="G65" s="3">
-        <v>45849</v>
+        <v>45852</v>
       </c>
       <c r="H65" s="3">
-        <v>45882</v>
+        <v>45867</v>
       </c>
       <c r="I65" s="3">
-        <v>45916</v>
+        <v>45922</v>
       </c>
       <c r="J65" t="s">
         <v>2</v>
@@ -3558,7 +3540,7 @@
         <v>1</v>
       </c>
       <c r="L65" s="3">
-        <v>45849</v>
+        <v>45852</v>
       </c>
     </row>
     <row r="66" spans="1:12" x14ac:dyDescent="0.25">
@@ -3566,7 +3548,7 @@
         <v>0</v>
       </c>
       <c r="B66" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C66" s="2">
         <v>1</v>
@@ -3575,28 +3557,28 @@
         <v>0</v>
       </c>
       <c r="E66" t="s">
-        <v>141</v>
+        <v>98</v>
       </c>
       <c r="F66" t="s">
-        <v>142</v>
+        <v>99</v>
       </c>
       <c r="G66" s="3">
-        <v>45849</v>
+        <v>45860</v>
       </c>
       <c r="H66" s="3">
         <v>45880</v>
       </c>
       <c r="I66" s="3">
-        <v>45910</v>
+        <v>45919</v>
       </c>
       <c r="J66" t="s">
-        <v>2</v>
+        <v>143</v>
       </c>
       <c r="K66" t="s">
         <v>1</v>
       </c>
       <c r="L66" s="3">
-        <v>45849</v>
+        <v>45860</v>
       </c>
     </row>
     <row r="67" spans="1:12" x14ac:dyDescent="0.25">
@@ -3613,19 +3595,19 @@
         <v>0</v>
       </c>
       <c r="E67" t="s">
-        <v>120</v>
+        <v>25</v>
       </c>
       <c r="F67" t="s">
-        <v>121</v>
+        <v>26</v>
       </c>
       <c r="G67" s="3">
-        <v>45852</v>
+        <v>45861</v>
       </c>
       <c r="H67" s="3">
-        <v>45867</v>
+        <v>45887</v>
       </c>
       <c r="I67" s="3">
-        <v>45922</v>
+        <v>45926</v>
       </c>
       <c r="J67" t="s">
         <v>2</v>
@@ -3634,7 +3616,7 @@
         <v>1</v>
       </c>
       <c r="L67" s="3">
-        <v>45852</v>
+        <v>45861</v>
       </c>
     </row>
     <row r="68" spans="1:12" x14ac:dyDescent="0.25">
@@ -3651,28 +3633,28 @@
         <v>0</v>
       </c>
       <c r="E68" t="s">
-        <v>101</v>
+        <v>25</v>
       </c>
       <c r="F68" t="s">
-        <v>102</v>
+        <v>26</v>
       </c>
       <c r="G68" s="3">
-        <v>45860</v>
+        <v>45861</v>
       </c>
       <c r="H68" s="3">
-        <v>45880</v>
+        <v>45883</v>
       </c>
       <c r="I68" s="3">
-        <v>45919</v>
+        <v>45912</v>
       </c>
       <c r="J68" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="K68" t="s">
         <v>1</v>
       </c>
       <c r="L68" s="3">
-        <v>45860</v>
+        <v>45861</v>
       </c>
     </row>
     <row r="69" spans="1:12" x14ac:dyDescent="0.25">
@@ -3680,31 +3662,31 @@
         <v>0</v>
       </c>
       <c r="B69" t="s">
+        <v>146</v>
+      </c>
+      <c r="C69" s="2">
+        <v>1</v>
+      </c>
+      <c r="D69" s="2">
+        <v>0</v>
+      </c>
+      <c r="E69" t="s">
         <v>147</v>
       </c>
-      <c r="C69" s="2">
-        <v>1</v>
-      </c>
-      <c r="D69" s="2">
-        <v>0</v>
-      </c>
-      <c r="E69" t="s">
-        <v>28</v>
-      </c>
       <c r="F69" t="s">
-        <v>29</v>
+        <v>148</v>
       </c>
       <c r="G69" s="3">
         <v>45861</v>
       </c>
       <c r="H69" s="3">
-        <v>45887</v>
+        <v>45996</v>
       </c>
       <c r="I69" s="3">
-        <v>45926</v>
+        <v>46085</v>
       </c>
       <c r="J69" t="s">
-        <v>2</v>
+        <v>149</v>
       </c>
       <c r="K69" t="s">
         <v>1</v>
@@ -3718,7 +3700,7 @@
         <v>0</v>
       </c>
       <c r="B70" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C70" s="2">
         <v>1</v>
@@ -3727,28 +3709,28 @@
         <v>0</v>
       </c>
       <c r="E70" t="s">
-        <v>28</v>
+        <v>131</v>
       </c>
       <c r="F70" t="s">
-        <v>29</v>
+        <v>132</v>
       </c>
       <c r="G70" s="3">
-        <v>45861</v>
+        <v>45866</v>
       </c>
       <c r="H70" s="3">
-        <v>45883</v>
+        <v>45880</v>
       </c>
       <c r="I70" s="3">
-        <v>45912</v>
+        <v>45910</v>
       </c>
       <c r="J70" t="s">
-        <v>146</v>
+        <v>2</v>
       </c>
       <c r="K70" t="s">
         <v>1</v>
       </c>
       <c r="L70" s="3">
-        <v>45861</v>
+        <v>45866</v>
       </c>
     </row>
     <row r="71" spans="1:12" x14ac:dyDescent="0.25">
@@ -3756,7 +3738,7 @@
         <v>0</v>
       </c>
       <c r="B71" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C71" s="2">
         <v>1</v>
@@ -3765,19 +3747,19 @@
         <v>0</v>
       </c>
       <c r="E71" t="s">
-        <v>150</v>
+        <v>12</v>
       </c>
       <c r="F71" t="s">
-        <v>151</v>
+        <v>13</v>
       </c>
       <c r="G71" s="3">
-        <v>45861</v>
+        <v>45870</v>
       </c>
       <c r="H71" s="3">
-        <v>45996</v>
+        <v>45987</v>
       </c>
       <c r="I71" s="3">
-        <v>46085</v>
+        <v>46055</v>
       </c>
       <c r="J71" t="s">
         <v>152</v>
@@ -3786,7 +3768,7 @@
         <v>1</v>
       </c>
       <c r="L71" s="3">
-        <v>45861</v>
+        <v>45870</v>
       </c>
     </row>
     <row r="72" spans="1:12" x14ac:dyDescent="0.25">
@@ -3803,28 +3785,28 @@
         <v>0</v>
       </c>
       <c r="E72" t="s">
-        <v>134</v>
+        <v>22</v>
       </c>
       <c r="F72" t="s">
-        <v>135</v>
+        <v>23</v>
       </c>
       <c r="G72" s="3">
-        <v>45866</v>
+        <v>45876</v>
       </c>
       <c r="H72" s="3">
-        <v>45880</v>
+        <v>45877</v>
       </c>
       <c r="I72" s="3">
         <v>45910</v>
       </c>
       <c r="J72" t="s">
-        <v>2</v>
+        <v>143</v>
       </c>
       <c r="K72" t="s">
         <v>1</v>
       </c>
       <c r="L72" s="3">
-        <v>45866</v>
+        <v>45875</v>
       </c>
     </row>
     <row r="73" spans="1:12" x14ac:dyDescent="0.25">
@@ -3841,28 +3823,28 @@
         <v>0</v>
       </c>
       <c r="E73" t="s">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="F73" t="s">
-        <v>13</v>
+        <v>35</v>
       </c>
       <c r="G73" s="3">
-        <v>45870</v>
+        <v>45876</v>
       </c>
       <c r="H73" s="3">
-        <v>45987</v>
+        <v>45891</v>
       </c>
       <c r="I73" s="3">
-        <v>46055</v>
+        <v>45917</v>
       </c>
       <c r="J73" t="s">
-        <v>155</v>
+        <v>143</v>
       </c>
       <c r="K73" t="s">
         <v>1</v>
       </c>
       <c r="L73" s="3">
-        <v>45870</v>
+        <v>45876</v>
       </c>
     </row>
     <row r="74" spans="1:12" x14ac:dyDescent="0.25">
@@ -3870,37 +3852,37 @@
         <v>0</v>
       </c>
       <c r="B74" t="s">
+        <v>155</v>
+      </c>
+      <c r="C74" s="2">
+        <v>1</v>
+      </c>
+      <c r="D74" s="2">
+        <v>0</v>
+      </c>
+      <c r="E74" t="s">
         <v>156</v>
       </c>
-      <c r="C74" s="2">
-        <v>1</v>
-      </c>
-      <c r="D74" s="2">
-        <v>0</v>
-      </c>
-      <c r="E74" t="s">
-        <v>25</v>
-      </c>
       <c r="F74" t="s">
-        <v>26</v>
+        <v>157</v>
       </c>
       <c r="G74" s="3">
         <v>45876</v>
       </c>
       <c r="H74" s="3">
-        <v>45877</v>
+        <v>45961</v>
       </c>
       <c r="I74" s="3">
-        <v>45910</v>
+        <v>45994</v>
       </c>
       <c r="J74" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="K74" t="s">
         <v>1</v>
       </c>
       <c r="L74" s="3">
-        <v>45875</v>
+        <v>45876</v>
       </c>
     </row>
     <row r="75" spans="1:12" x14ac:dyDescent="0.25">
@@ -3908,7 +3890,7 @@
         <v>0</v>
       </c>
       <c r="B75" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C75" s="2">
         <v>1</v>
@@ -3917,28 +3899,28 @@
         <v>0</v>
       </c>
       <c r="E75" t="s">
-        <v>37</v>
+        <v>19</v>
       </c>
       <c r="F75" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="G75" s="3">
-        <v>45876</v>
+        <v>45880</v>
       </c>
       <c r="H75" s="3">
-        <v>45891</v>
+        <v>45925</v>
       </c>
       <c r="I75" s="3">
-        <v>45917</v>
+        <v>46021</v>
       </c>
       <c r="J75" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="K75" t="s">
         <v>1</v>
       </c>
       <c r="L75" s="3">
-        <v>45876</v>
+        <v>45880</v>
       </c>
     </row>
     <row r="76" spans="1:12" x14ac:dyDescent="0.25">
@@ -3946,7 +3928,7 @@
         <v>0</v>
       </c>
       <c r="B76" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C76" s="2">
         <v>1</v>
@@ -3955,28 +3937,28 @@
         <v>0</v>
       </c>
       <c r="E76" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="F76" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="G76" s="3">
-        <v>45876</v>
+        <v>45880</v>
       </c>
       <c r="H76" s="3">
-        <v>45961</v>
+        <v>45887</v>
       </c>
       <c r="I76" s="3">
-        <v>45994</v>
+        <v>45938</v>
       </c>
       <c r="J76" t="s">
-        <v>155</v>
+        <v>143</v>
       </c>
       <c r="K76" t="s">
         <v>1</v>
       </c>
       <c r="L76" s="3">
-        <v>45876</v>
+        <v>45880</v>
       </c>
     </row>
     <row r="77" spans="1:12" x14ac:dyDescent="0.25">
@@ -3984,7 +3966,7 @@
         <v>0</v>
       </c>
       <c r="B77" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C77" s="2">
         <v>1</v>
@@ -3993,22 +3975,22 @@
         <v>0</v>
       </c>
       <c r="E77" t="s">
-        <v>22</v>
+        <v>50</v>
       </c>
       <c r="F77" t="s">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="G77" s="3">
         <v>45880</v>
       </c>
       <c r="H77" s="3">
-        <v>45925</v>
+        <v>45888</v>
       </c>
       <c r="I77" s="3">
-        <v>46021</v>
+        <v>45922</v>
       </c>
       <c r="J77" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="K77" t="s">
         <v>1</v>
@@ -4022,7 +4004,7 @@
         <v>0</v>
       </c>
       <c r="B78" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C78" s="2">
         <v>1</v>
@@ -4031,28 +4013,28 @@
         <v>0</v>
       </c>
       <c r="E78" t="s">
-        <v>159</v>
+        <v>127</v>
       </c>
       <c r="F78" t="s">
-        <v>160</v>
+        <v>128</v>
       </c>
       <c r="G78" s="3">
-        <v>45880</v>
+        <v>45882</v>
       </c>
       <c r="H78" s="3">
-        <v>45887</v>
+        <v>45918</v>
       </c>
       <c r="I78" s="3">
-        <v>45938</v>
+        <v>45945</v>
       </c>
       <c r="J78" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="K78" t="s">
         <v>1</v>
       </c>
       <c r="L78" s="3">
-        <v>45880</v>
+        <v>45882</v>
       </c>
     </row>
     <row r="79" spans="1:12" x14ac:dyDescent="0.25">
@@ -4060,7 +4042,7 @@
         <v>0</v>
       </c>
       <c r="B79" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C79" s="2">
         <v>1</v>
@@ -4075,22 +4057,22 @@
         <v>54</v>
       </c>
       <c r="G79" s="3">
-        <v>45880</v>
+        <v>45882</v>
       </c>
       <c r="H79" s="3">
-        <v>45888</v>
+        <v>45896</v>
       </c>
       <c r="I79" s="3">
-        <v>45922</v>
+        <v>45923</v>
       </c>
       <c r="J79" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="K79" t="s">
         <v>1</v>
       </c>
       <c r="L79" s="3">
-        <v>45880</v>
+        <v>45882</v>
       </c>
     </row>
     <row r="80" spans="1:12" x14ac:dyDescent="0.25">
@@ -4098,37 +4080,37 @@
         <v>0</v>
       </c>
       <c r="B80" t="s">
+        <v>163</v>
+      </c>
+      <c r="C80" s="2">
+        <v>1</v>
+      </c>
+      <c r="D80" s="2">
+        <v>0</v>
+      </c>
+      <c r="E80" t="s">
         <v>164</v>
       </c>
-      <c r="C80" s="2">
-        <v>1</v>
-      </c>
-      <c r="D80" s="2">
-        <v>0</v>
-      </c>
-      <c r="E80" t="s">
-        <v>130</v>
-      </c>
       <c r="F80" t="s">
-        <v>131</v>
+        <v>165</v>
       </c>
       <c r="G80" s="3">
-        <v>45882</v>
+        <v>45884</v>
       </c>
       <c r="H80" s="3">
-        <v>45918</v>
+        <v>45930</v>
       </c>
       <c r="I80" s="3">
-        <v>45945</v>
+        <v>45959</v>
       </c>
       <c r="J80" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="K80" t="s">
         <v>1</v>
       </c>
       <c r="L80" s="3">
-        <v>45882</v>
+        <v>45884</v>
       </c>
     </row>
     <row r="81" spans="1:12" x14ac:dyDescent="0.25">
@@ -4136,7 +4118,7 @@
         <v>0</v>
       </c>
       <c r="B81" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C81" s="2">
         <v>1</v>
@@ -4145,28 +4127,28 @@
         <v>0</v>
       </c>
       <c r="E81" t="s">
-        <v>56</v>
+        <v>127</v>
       </c>
       <c r="F81" t="s">
-        <v>57</v>
+        <v>128</v>
       </c>
       <c r="G81" s="3">
-        <v>45882</v>
+        <v>45884</v>
       </c>
       <c r="H81" s="3">
-        <v>45896</v>
+        <v>45971</v>
       </c>
       <c r="I81" s="3">
-        <v>45923</v>
+        <v>45994</v>
       </c>
       <c r="J81" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="K81" t="s">
         <v>1</v>
       </c>
       <c r="L81" s="3">
-        <v>45882</v>
+        <v>45884</v>
       </c>
     </row>
     <row r="82" spans="1:12" x14ac:dyDescent="0.25">
@@ -4174,7 +4156,7 @@
         <v>0</v>
       </c>
       <c r="B82" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C82" s="2">
         <v>1</v>
@@ -4183,22 +4165,22 @@
         <v>0</v>
       </c>
       <c r="E82" t="s">
-        <v>167</v>
+        <v>127</v>
       </c>
       <c r="F82" t="s">
-        <v>168</v>
+        <v>128</v>
       </c>
       <c r="G82" s="3">
         <v>45884</v>
       </c>
       <c r="H82" s="3">
-        <v>45930</v>
+        <v>45971</v>
       </c>
       <c r="I82" s="3">
-        <v>45959</v>
+        <v>45994</v>
       </c>
       <c r="J82" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="K82" t="s">
         <v>1</v>
@@ -4212,7 +4194,7 @@
         <v>0</v>
       </c>
       <c r="B83" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C83" s="2">
         <v>1</v>
@@ -4221,10 +4203,10 @@
         <v>0</v>
       </c>
       <c r="E83" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="F83" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="G83" s="3">
         <v>45884</v>
@@ -4236,7 +4218,7 @@
         <v>45994</v>
       </c>
       <c r="J83" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="K83" t="s">
         <v>1</v>
@@ -4250,7 +4232,7 @@
         <v>0</v>
       </c>
       <c r="B84" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C84" s="2">
         <v>1</v>
@@ -4259,10 +4241,10 @@
         <v>0</v>
       </c>
       <c r="E84" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="F84" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="G84" s="3">
         <v>45884</v>
@@ -4274,7 +4256,7 @@
         <v>45994</v>
       </c>
       <c r="J84" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="K84" t="s">
         <v>1</v>
@@ -4288,7 +4270,7 @@
         <v>0</v>
       </c>
       <c r="B85" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C85" s="2">
         <v>1</v>
@@ -4297,22 +4279,22 @@
         <v>0</v>
       </c>
       <c r="E85" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="F85" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="G85" s="3">
         <v>45884</v>
       </c>
       <c r="H85" s="3">
-        <v>45971</v>
+        <v>45958</v>
       </c>
       <c r="I85" s="3">
-        <v>45994</v>
+        <v>45981</v>
       </c>
       <c r="J85" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="K85" t="s">
         <v>1</v>
@@ -4326,7 +4308,7 @@
         <v>0</v>
       </c>
       <c r="B86" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C86" s="2">
         <v>1</v>
@@ -4335,22 +4317,22 @@
         <v>0</v>
       </c>
       <c r="E86" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="F86" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="G86" s="3">
         <v>45884</v>
       </c>
       <c r="H86" s="3">
-        <v>45971</v>
+        <v>45958</v>
       </c>
       <c r="I86" s="3">
-        <v>45994</v>
+        <v>45981</v>
       </c>
       <c r="J86" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="K86" t="s">
         <v>1</v>
@@ -4364,7 +4346,7 @@
         <v>0</v>
       </c>
       <c r="B87" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C87" s="2">
         <v>1</v>
@@ -4373,10 +4355,10 @@
         <v>0</v>
       </c>
       <c r="E87" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="F87" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="G87" s="3">
         <v>45884</v>
@@ -4388,7 +4370,7 @@
         <v>45981</v>
       </c>
       <c r="J87" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="K87" t="s">
         <v>1</v>
@@ -4402,7 +4384,7 @@
         <v>0</v>
       </c>
       <c r="B88" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C88" s="2">
         <v>1</v>
@@ -4411,10 +4393,10 @@
         <v>0</v>
       </c>
       <c r="E88" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="F88" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="G88" s="3">
         <v>45884</v>
@@ -4426,7 +4408,7 @@
         <v>45981</v>
       </c>
       <c r="J88" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="K88" t="s">
         <v>1</v>
@@ -4440,37 +4422,37 @@
         <v>0</v>
       </c>
       <c r="B89" t="s">
+        <v>174</v>
+      </c>
+      <c r="C89" s="2">
+        <v>1</v>
+      </c>
+      <c r="D89" s="2">
+        <v>0</v>
+      </c>
+      <c r="E89" t="s">
         <v>175</v>
       </c>
-      <c r="C89" s="2">
-        <v>1</v>
-      </c>
-      <c r="D89" s="2">
-        <v>0</v>
-      </c>
-      <c r="E89" t="s">
-        <v>130</v>
-      </c>
       <c r="F89" t="s">
-        <v>131</v>
+        <v>176</v>
       </c>
       <c r="G89" s="3">
-        <v>45884</v>
+        <v>45887</v>
       </c>
       <c r="H89" s="3">
-        <v>45958</v>
+        <v>45999</v>
       </c>
       <c r="I89" s="3">
-        <v>45981</v>
+        <v>46084</v>
       </c>
       <c r="J89" t="s">
-        <v>155</v>
+        <v>177</v>
       </c>
       <c r="K89" t="s">
         <v>1</v>
       </c>
       <c r="L89" s="3">
-        <v>45884</v>
+        <v>45887</v>
       </c>
     </row>
     <row r="90" spans="1:12" x14ac:dyDescent="0.25">
@@ -4478,7 +4460,7 @@
         <v>0</v>
       </c>
       <c r="B90" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="C90" s="2">
         <v>1</v>
@@ -4487,28 +4469,28 @@
         <v>0</v>
       </c>
       <c r="E90" t="s">
-        <v>130</v>
+        <v>34</v>
       </c>
       <c r="F90" t="s">
-        <v>131</v>
+        <v>35</v>
       </c>
       <c r="G90" s="3">
-        <v>45884</v>
+        <v>45891</v>
       </c>
       <c r="H90" s="3">
-        <v>45958</v>
+        <v>45905</v>
       </c>
       <c r="I90" s="3">
-        <v>45981</v>
+        <v>45926</v>
       </c>
       <c r="J90" t="s">
-        <v>155</v>
+        <v>179</v>
       </c>
       <c r="K90" t="s">
         <v>1</v>
       </c>
       <c r="L90" s="3">
-        <v>45884</v>
+        <v>45890</v>
       </c>
     </row>
     <row r="91" spans="1:12" x14ac:dyDescent="0.25">
@@ -4516,7 +4498,7 @@
         <v>0</v>
       </c>
       <c r="B91" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C91" s="2">
         <v>1</v>
@@ -4525,28 +4507,28 @@
         <v>0</v>
       </c>
       <c r="E91" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="F91" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="G91" s="3">
-        <v>45887</v>
+        <v>45891</v>
       </c>
       <c r="H91" s="3">
-        <v>45999</v>
+        <v>45895</v>
       </c>
       <c r="I91" s="3">
-        <v>46084</v>
+        <v>45916</v>
       </c>
       <c r="J91" t="s">
-        <v>180</v>
+        <v>143</v>
       </c>
       <c r="K91" t="s">
         <v>1</v>
       </c>
       <c r="L91" s="3">
-        <v>45887</v>
+        <v>45891</v>
       </c>
     </row>
     <row r="92" spans="1:12" x14ac:dyDescent="0.25">
@@ -4554,37 +4536,37 @@
         <v>0</v>
       </c>
       <c r="B92" t="s">
+        <v>183</v>
+      </c>
+      <c r="C92" s="2">
+        <v>1</v>
+      </c>
+      <c r="D92" s="2">
+        <v>0</v>
+      </c>
+      <c r="E92" t="s">
         <v>181</v>
       </c>
-      <c r="C92" s="2">
-        <v>1</v>
-      </c>
-      <c r="D92" s="2">
-        <v>0</v>
-      </c>
-      <c r="E92" t="s">
-        <v>37</v>
-      </c>
       <c r="F92" t="s">
-        <v>38</v>
+        <v>182</v>
       </c>
       <c r="G92" s="3">
         <v>45891</v>
       </c>
       <c r="H92" s="3">
-        <v>45905</v>
+        <v>45891</v>
       </c>
       <c r="I92" s="3">
-        <v>45926</v>
+        <v>45915</v>
       </c>
       <c r="J92" t="s">
-        <v>182</v>
+        <v>143</v>
       </c>
       <c r="K92" t="s">
         <v>1</v>
       </c>
       <c r="L92" s="3">
-        <v>45890</v>
+        <v>45891</v>
       </c>
     </row>
     <row r="93" spans="1:12" x14ac:dyDescent="0.25">
@@ -4592,7 +4574,7 @@
         <v>0</v>
       </c>
       <c r="B93" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C93" s="2">
         <v>1</v>
@@ -4601,28 +4583,28 @@
         <v>0</v>
       </c>
       <c r="E93" t="s">
-        <v>184</v>
+        <v>22</v>
       </c>
       <c r="F93" t="s">
-        <v>185</v>
+        <v>23</v>
       </c>
       <c r="G93" s="3">
-        <v>45891</v>
+        <v>45901</v>
       </c>
       <c r="H93" s="3">
-        <v>45895</v>
+        <v>45902</v>
       </c>
       <c r="I93" s="3">
-        <v>45916</v>
+        <v>45931</v>
       </c>
       <c r="J93" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="K93" t="s">
         <v>1</v>
       </c>
       <c r="L93" s="3">
-        <v>45891</v>
+        <v>45901</v>
       </c>
     </row>
     <row r="94" spans="1:12" x14ac:dyDescent="0.25">
@@ -4630,37 +4612,37 @@
         <v>0</v>
       </c>
       <c r="B94" t="s">
+        <v>185</v>
+      </c>
+      <c r="C94" s="2">
+        <v>1</v>
+      </c>
+      <c r="D94" s="2">
+        <v>0</v>
+      </c>
+      <c r="E94" t="s">
+        <v>4</v>
+      </c>
+      <c r="F94" t="s">
+        <v>5</v>
+      </c>
+      <c r="G94" s="3">
+        <v>45901</v>
+      </c>
+      <c r="H94" s="3">
+        <v>45968</v>
+      </c>
+      <c r="I94" s="3">
+        <v>45993</v>
+      </c>
+      <c r="J94" t="s">
         <v>186</v>
       </c>
-      <c r="C94" s="2">
-        <v>1</v>
-      </c>
-      <c r="D94" s="2">
-        <v>0</v>
-      </c>
-      <c r="E94" t="s">
-        <v>184</v>
-      </c>
-      <c r="F94" t="s">
-        <v>185</v>
-      </c>
-      <c r="G94" s="3">
-        <v>45891</v>
-      </c>
-      <c r="H94" s="3">
-        <v>45891</v>
-      </c>
-      <c r="I94" s="3">
-        <v>45915</v>
-      </c>
-      <c r="J94" t="s">
-        <v>146</v>
-      </c>
       <c r="K94" t="s">
         <v>1</v>
       </c>
       <c r="L94" s="3">
-        <v>45891</v>
+        <v>45901</v>
       </c>
     </row>
     <row r="95" spans="1:12" x14ac:dyDescent="0.25">
@@ -4677,22 +4659,22 @@
         <v>0</v>
       </c>
       <c r="E95" t="s">
-        <v>25</v>
+        <v>188</v>
       </c>
       <c r="F95" t="s">
-        <v>26</v>
+        <v>189</v>
       </c>
       <c r="G95" s="3">
         <v>45901</v>
       </c>
       <c r="H95" s="3">
-        <v>45902</v>
+        <v>46055</v>
       </c>
       <c r="I95" s="3">
-        <v>45931</v>
+        <v>46140</v>
       </c>
       <c r="J95" t="s">
-        <v>146</v>
+        <v>186</v>
       </c>
       <c r="K95" t="s">
         <v>1</v>
@@ -4701,85 +4683,9 @@
         <v>45901</v>
       </c>
     </row>
-    <row r="96" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A96" t="s">
-        <v>0</v>
-      </c>
-      <c r="B96" t="s">
-        <v>188</v>
-      </c>
-      <c r="C96" s="2">
-        <v>1</v>
-      </c>
-      <c r="D96" s="2">
-        <v>0</v>
-      </c>
-      <c r="E96" t="s">
-        <v>4</v>
-      </c>
-      <c r="F96" t="s">
-        <v>5</v>
-      </c>
-      <c r="G96" s="3">
-        <v>45901</v>
-      </c>
-      <c r="H96" s="3">
-        <v>45968</v>
-      </c>
-      <c r="I96" s="3">
-        <v>45993</v>
-      </c>
-      <c r="J96" t="s">
-        <v>189</v>
-      </c>
-      <c r="K96" t="s">
-        <v>1</v>
-      </c>
-      <c r="L96" s="3">
-        <v>45901</v>
-      </c>
-    </row>
-    <row r="97" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A97" t="s">
-        <v>0</v>
-      </c>
-      <c r="B97" t="s">
-        <v>190</v>
-      </c>
-      <c r="C97" s="2">
-        <v>1</v>
-      </c>
-      <c r="D97" s="2">
-        <v>0</v>
-      </c>
-      <c r="E97" t="s">
-        <v>191</v>
-      </c>
-      <c r="F97" t="s">
-        <v>192</v>
-      </c>
-      <c r="G97" s="3">
-        <v>45901</v>
-      </c>
-      <c r="H97" s="3">
-        <v>46055</v>
-      </c>
-      <c r="I97" s="3">
-        <v>46140</v>
-      </c>
-      <c r="J97" t="s">
-        <v>189</v>
-      </c>
-      <c r="K97" t="s">
-        <v>1</v>
-      </c>
-      <c r="L97" s="3">
-        <v>45901</v>
-      </c>
-    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L97">
-    <sortCondition ref="B2:B97"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L95">
+    <sortCondition ref="B2:B95"/>
   </sortState>
   <phoneticPr fontId="0" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>